<commit_message>
Agente ADS: plan B de Juan (visibilidad con tope de pérdida semanal)
Juan (18/10): 'Hagamos el plan B', 'Yo pausé pinza V2', 'Haz el cupón'.
- directivas.json -> visibilidad: pujas fijadas a 0,40 € en lo que ha
  vendido (automática substitutes, exacta 'soporte teléfono coche',
  B0F3J3QHD7, B08N4KR6PK, B09P3SZB6P) hasta el 02/12, con tope de
  10 € de pérdida por semana; al llegar, el plan se para hasta el lunes.
- directivas.py/agente.py: el motor aplica el plan y sustituye sus
  propias pujas para esos elementos; tests nuevos.
- bulk_cambios_2026-10-18.xlsx con las 4 subidas; cupón de la pinza
  propuesto (5 %, 20/11-02/12) en ESTRATEGIA.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8zFsXd31MYxmY7hRPcJU8
</commit_message>
<xml_diff>
--- a/salidas/2026-10-18/ficha_datos_2026-10-18.xlsx
+++ b/salidas/2026-10-18/ficha_datos_2026-10-18.xlsx
@@ -1108,7 +1108,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>moviles</t>
+          <t>sujeta</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1124,7 +1124,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>sujeta</t>
+          <t>moviles</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1619,7 +1619,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>holder</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1635,7 +1635,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>holder</t>
+          <t>car</t>
         </is>
       </c>
       <c r="B15" t="n">

</xml_diff>